<commit_message>
Clarify quasi-rent margin semantics: operating costs only, depreciation charged in user cost (adversarial review catch). Comment-only; no parameter values changed, no restatement triggered
</commit_message>
<xml_diff>
--- a/docs/data/rot-methodology.xlsx
+++ b/docs/data/rot-methodology.xlsx
@@ -572,7 +572,7 @@
     <t xml:space="preserve">AI-attributable revenue ($bn/yr)</t>
   </si>
   <si>
-    <t xml:space="preserve">ILLUSTRATIVE - tiered T1/T2/T3 assembly in pipeline</t>
+    <t xml:space="preserve">margin = revenue net of OPERATING costs only; depreciation is charged in the user cost (row 15), never netted here - double-counting guard</t>
   </si>
   <si>
     <t xml:space="preserve">Quasi-rents LOW ($bn)</t>
@@ -606,7 +606,7 @@
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -646,6 +646,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -699,36 +706,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -987,68 +1002,68 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="84"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1071,271 +1086,271 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="46"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" s="1" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="F11" s="1" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" s="1" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1358,177 +1373,177 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="64"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>124</v>
       </c>
     </row>
@@ -1551,195 +1566,195 @@
   <dimension ref="A1:C26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="56"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="4" t="n">
         <v>4.45</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="4" t="n">
         <v>4.23</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="4" t="n">
         <v>0.18</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="4" t="n">
         <v>0.28</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="4" t="n">
         <v>0.025</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="4" t="n">
         <v>0.04</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="4" t="n">
         <v>0.3</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="4" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="4" t="n">
         <v>0.7</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>157</v>
       </c>
     </row>
@@ -1762,257 +1777,257 @@
   <dimension ref="A1:E22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="4" t="n">
         <v>97</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="4" t="n">
         <v>170</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="6" t="n">
         <f aca="false">B3/C3</f>
         <v>0.570588235294118</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="4" t="n">
         <v>110</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="4" t="n">
         <v>174</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="6" t="n">
         <f aca="false">B4/C4</f>
         <v>0.632183908045977</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="4" t="n">
         <v>124</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="6" t="n">
         <f aca="false">B5/C5</f>
         <v>0.612903225806452</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="4" t="n">
         <v>151</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="4" t="n">
         <v>149</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="6" t="n">
         <f aca="false">B6/C6</f>
         <v>1.01342281879195</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="6" t="n">
         <f aca="false">B7/C7</f>
         <v>2</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="4" t="n">
         <v>600</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="4" t="n">
         <v>250</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="4" t="n">
         <v>150</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <f aca="false">('Assumptions v1'!B3+'Assumptions v1'!B4)/100</f>
         <v>0.0868</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="7" t="n">
         <f aca="false">(B14+'Assumptions v1'!B8)*B11+(B14+'Assumptions v1'!B12)*B12+(B14+'Assumptions v1'!B16)*B13</f>
         <v>267.05</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="8" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <f aca="false">B18*'Assumptions v1'!B19</f>
         <v>18</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="1" t="n">
         <f aca="false">B18*'Assumptions v1'!B21</f>
         <v>42</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="1" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="9" t="n">
         <f aca="false">B19/B15</f>
         <v>0.0674031080322037</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B22" s="9" t="n">
         <f aca="false">B20/B15</f>
         <v>0.157273918741809</v>
       </c>

</xml_diff>